<commit_message>
stepper motor controller circuit moredevelopment and started the programming
</commit_message>
<xml_diff>
--- a/stepper_motor_controller/BOM.xlsx
+++ b/stepper_motor_controller/BOM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -49,22 +49,40 @@
     <t xml:space="preserve">5*3.5</t>
   </si>
   <si>
-    <t xml:space="preserve">Arduino Nano</t>
+    <t xml:space="preserve">STC8H8K64U</t>
   </si>
   <si>
     <t xml:space="preserve">RAM</t>
   </si>
   <si>
-    <t xml:space="preserve">Pin Headers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ULN2803</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JST 5 pin Female</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capacitor</t>
+    <t xml:space="preserve">SOP16 Breakout </t>
+  </si>
+  <si>
+    <t xml:space="preserve">UGE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LM317</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heat sink</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rotary Encoder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">free electronics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OLED 1.4inch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TMC2209</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JST 4P Female</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terminal 2Pin</t>
   </si>
   <si>
     <t xml:space="preserve">**</t>
@@ -96,7 +114,6 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -119,14 +136,12 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -412,7 +427,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -501,8 +516,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="10.50390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
@@ -510,10 +525,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="5.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="5.99"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -536,7 +551,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="n">
         <v>1</v>
       </c>
@@ -558,7 +573,7 @@
       </c>
       <c r="G2" s="11"/>
     </row>
-    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
@@ -566,21 +581,22 @@
         <v>9</v>
       </c>
       <c r="C3" s="13" t="n">
-        <v>275</v>
+        <f aca="false">60+0.14*60</f>
+        <v>68.4</v>
       </c>
       <c r="D3" s="5" t="n">
         <v>1</v>
       </c>
       <c r="E3" s="14" t="n">
         <f aca="false">C3*D3</f>
-        <v>275</v>
+        <v>68.4</v>
       </c>
       <c r="F3" s="15"/>
       <c r="G3" s="16" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="n">
         <v>3</v>
       </c>
@@ -588,165 +604,229 @@
         <v>11</v>
       </c>
       <c r="C4" s="13" t="n">
-        <v>2.5</v>
+        <v>35</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" s="14" t="n">
         <f aca="false">C4*D4</f>
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="F4" s="15"/>
       <c r="G4" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5"/>
+      <c r="B5" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="13"/>
+      <c r="D5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="14"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="16"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5"/>
+      <c r="B6" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="13"/>
+      <c r="D6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="14"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="16"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="13" t="n">
-        <v>13</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="14" t="n">
-        <f aca="false">C5*D5</f>
-        <v>13</v>
-      </c>
-      <c r="F5" s="15"/>
-      <c r="G5" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="13" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="14" t="n">
-        <f aca="false">C6*D6</f>
-        <v>2.5</v>
-      </c>
-      <c r="F6" s="15"/>
-      <c r="G6" s="17" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="n">
-        <v>6</v>
-      </c>
       <c r="B7" s="12" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C7" s="13" t="n">
-        <v>1.5</v>
+        <v>60</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="14" t="n">
         <f aca="false">C7*D7</f>
-        <v>1.5</v>
+        <v>60</v>
       </c>
       <c r="F7" s="15"/>
-      <c r="G7" s="17" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="14"/>
+      <c r="G7" s="16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="13" t="n">
+        <v>350</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="14" t="n">
+        <f aca="false">C8*D8</f>
+        <v>350</v>
+      </c>
       <c r="F8" s="15"/>
-      <c r="G8" s="16"/>
-    </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
-        <v>15</v>
+      <c r="G8" s="17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="n">
+        <v>6</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C9" s="13" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="14" t="n">
         <f aca="false">C9*D9</f>
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="F9" s="15"/>
-      <c r="G9" s="16"/>
-    </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="14"/>
-      <c r="G10" s="16"/>
-    </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="20" t="n">
-        <v>400</v>
-      </c>
-      <c r="D11" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="21" t="n">
+      <c r="G9" s="17" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="14" t="n">
+        <f aca="false">C10*D10</f>
+        <v>2</v>
+      </c>
+      <c r="F10" s="15"/>
+      <c r="G10" s="17"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="14" t="n">
         <f aca="false">C11*D11</f>
-        <v>400</v>
+        <v>3</v>
       </c>
       <c r="F11" s="15"/>
-      <c r="G11" s="16"/>
-    </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G11" s="17"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
-      <c r="B12" s="22"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="25"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="14"/>
       <c r="F12" s="15"/>
       <c r="G12" s="16"/>
     </row>
-    <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1"/>
-      <c r="B13" s="26" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="27"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="2" t="n">
-        <f aca="false">SUM(E2:E12)</f>
-        <v>947</v>
-      </c>
-      <c r="F13" s="29"/>
-      <c r="G13" s="30"/>
+    <row r="13" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="13"/>
+      <c r="D13" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="14" t="n">
+        <f aca="false">C13*D13</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="15"/>
+      <c r="G13" s="16"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="14"/>
+      <c r="G14" s="16"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="21" t="n">
+        <f aca="false">C15*D15</f>
+        <v>0</v>
+      </c>
+      <c r="F15" s="15"/>
+      <c r="G15" s="16"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="16"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1"/>
+      <c r="B17" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="27"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="2" t="n">
+        <f aca="false">SUM(E2:E16)</f>
+        <v>818.4</v>
+      </c>
+      <c r="F17" s="29"/>
+      <c r="G17" s="30"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
huge progress in programming in stepper_motor_controller project
</commit_message>
<xml_diff>
--- a/stepper_motor_controller/BOM.xlsx
+++ b/stepper_motor_controller/BOM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -52,13 +52,7 @@
     <t xml:space="preserve">STC8H8K64U</t>
   </si>
   <si>
-    <t xml:space="preserve">RAM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOP16 Breakout </t>
-  </si>
-  <si>
-    <t xml:space="preserve">UGE</t>
+    <t xml:space="preserve">IC Socket DIP 28</t>
   </si>
   <si>
     <t xml:space="preserve">LM317</t>
@@ -67,13 +61,37 @@
     <t xml:space="preserve">Heat sink</t>
   </si>
   <si>
+    <t xml:space="preserve">Capacitors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">470uf and 10nf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">330, 220 and 100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Switch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pin Header 1x3</t>
+  </si>
+  <si>
     <t xml:space="preserve">rotary Encoder</t>
   </si>
   <si>
-    <t xml:space="preserve">free electronics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OLED 1.4inch</t>
+    <t xml:space="preserve">OLED 0.96inch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pin Header 1x6</t>
   </si>
   <si>
     <t xml:space="preserve">TMC2209</t>
@@ -114,6 +132,7 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -136,12 +155,14 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -374,8 +395,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -516,318 +541,459 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G1048576"/>
+  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="5.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="5.99"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="8" style="1" width="10.51"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="6" t="s">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="7" t="n">
+      <c r="C2" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="D2" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="9" t="n">
+      <c r="D2" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="10" t="n">
         <f aca="false">C2*D2</f>
         <v>50</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="11"/>
+      <c r="G2" s="12"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="13" t="n">
-        <f aca="false">60+0.14*60</f>
-        <v>68.4</v>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="14" t="n">
+      <c r="C3" s="14" t="n">
+        <f aca="false">81+0.14*81</f>
+        <v>92.34</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="15" t="n">
         <f aca="false">C3*D3</f>
-        <v>68.4</v>
-      </c>
-      <c r="F3" s="15"/>
-      <c r="G3" s="16" t="s">
+        <v>92.34</v>
+      </c>
+      <c r="F3" s="16"/>
+      <c r="G3" s="17"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="13" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="n">
+      <c r="C4" s="14" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="15" t="n">
+        <f aca="false">C4*D4</f>
+        <v>2.75</v>
+      </c>
+      <c r="F4" s="16"/>
+      <c r="G4" s="17"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="15" t="n">
+        <f aca="false">C5*D5</f>
+        <v>6</v>
+      </c>
+      <c r="F5" s="16"/>
+      <c r="G5" s="17"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <f aca="false">C6*D6</f>
+        <v>3.5</v>
+      </c>
+      <c r="F6" s="16"/>
+      <c r="G6" s="17"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <f aca="false">C7*D7</f>
+        <v>5</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="17"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="E8" s="15" t="n">
+        <f aca="false">C8*D8</f>
+        <v>3</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="17"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <f aca="false">C9*D9</f>
+        <v>1</v>
+      </c>
+      <c r="F9" s="16"/>
+      <c r="G9" s="17"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <f aca="false">C10*D10</f>
+        <v>2.25</v>
+      </c>
+      <c r="F10" s="16"/>
+      <c r="G10" s="17"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="15" t="n">
+        <f aca="false">C11*D11</f>
+        <v>1.5</v>
+      </c>
+      <c r="F11" s="16"/>
+      <c r="G11" s="17"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="C4" s="13" t="n">
-        <v>35</v>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="14" t="n">
-        <f aca="false">C4*D4</f>
-        <v>35</v>
-      </c>
-      <c r="F4" s="15"/>
-      <c r="G4" s="16" t="s">
+      <c r="B12" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <f aca="false">C12*D12</f>
+        <v>3</v>
+      </c>
+      <c r="F12" s="16"/>
+      <c r="G12" s="17"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="n">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="12" t="s">
+      <c r="B13" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="15" t="n">
+        <f aca="false">C13*D13</f>
+        <v>60</v>
+      </c>
+      <c r="F13" s="16"/>
+      <c r="G13" s="17"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="C5" s="13"/>
-      <c r="D5" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="14"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="16"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5"/>
-      <c r="B6" s="12" t="s">
+      <c r="B14" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>170</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <f aca="false">C14*D14</f>
+        <v>170</v>
+      </c>
+      <c r="F14" s="16"/>
+      <c r="G14" s="18"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="C6" s="13"/>
-      <c r="D6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="14"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="16"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="12" t="s">
+      <c r="B15" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <f aca="false">C15*D15</f>
+        <v>6</v>
+      </c>
+      <c r="F15" s="16"/>
+      <c r="G15" s="18"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="C7" s="13" t="n">
-        <v>60</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="14" t="n">
-        <f aca="false">C7*D7</f>
-        <v>60</v>
-      </c>
-      <c r="F7" s="15"/>
-      <c r="G7" s="16" t="s">
+      <c r="B16" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <f aca="false">C16*D16</f>
+        <v>250</v>
+      </c>
+      <c r="F16" s="16"/>
+      <c r="G16" s="18"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="n">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="12" t="s">
+      <c r="B17" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <f aca="false">C17*D17</f>
+        <v>1</v>
+      </c>
+      <c r="F17" s="16"/>
+      <c r="G17" s="18"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="C8" s="13" t="n">
-        <v>350</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="14" t="n">
-        <f aca="false">C8*D8</f>
-        <v>350</v>
-      </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="13" t="n">
-        <v>250</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="14" t="n">
-        <f aca="false">C9*D9</f>
-        <v>250</v>
-      </c>
-      <c r="F9" s="15"/>
-      <c r="G9" s="17" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="14" t="n">
-        <f aca="false">C10*D10</f>
-        <v>2</v>
-      </c>
-      <c r="F10" s="15"/>
-      <c r="G10" s="17"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="13" t="n">
+      <c r="B18" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="D11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="14" t="n">
-        <f aca="false">C11*D11</f>
+      <c r="D18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <f aca="false">C18*D18</f>
         <v>3</v>
       </c>
-      <c r="F11" s="15"/>
-      <c r="G11" s="17"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="16"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="C13" s="13"/>
-      <c r="D13" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="14" t="n">
-        <f aca="false">C13*D13</f>
+      <c r="F18" s="16"/>
+      <c r="G18" s="18"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" s="14"/>
+      <c r="D19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <f aca="false">C19*D19</f>
         <v>0</v>
       </c>
-      <c r="F13" s="15"/>
-      <c r="G13" s="16"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5"/>
-      <c r="B14" s="12"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="14"/>
-      <c r="G14" s="16"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" s="20" t="n">
+      <c r="F19" s="16"/>
+      <c r="G19" s="17"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="15"/>
+      <c r="G20" s="17"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="21" t="n">
-        <f aca="false">C15*D15</f>
+      <c r="D21" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="22" t="n">
+        <f aca="false">C21*D21</f>
         <v>0</v>
       </c>
-      <c r="F15" s="15"/>
-      <c r="G15" s="16"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="22"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="16"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1"/>
-      <c r="B17" s="26" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="27"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="2" t="n">
-        <f aca="false">SUM(E2:E16)</f>
-        <v>818.4</v>
-      </c>
-      <c r="F17" s="29"/>
-      <c r="G17" s="30"/>
-    </row>
+      <c r="F21" s="16"/>
+      <c r="G21" s="17"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="17"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2"/>
+      <c r="B23" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="28"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="3" t="n">
+        <f aca="false">SUM(E2:E22)</f>
+        <v>660.34</v>
+      </c>
+      <c r="F23" s="30"/>
+      <c r="G23" s="31"/>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
started keyboard emulator project and updated wind sensor code
</commit_message>
<xml_diff>
--- a/stepper_motor_controller/BOM.xlsx
+++ b/stepper_motor_controller/BOM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -103,6 +103,9 @@
     <t xml:space="preserve">Terminal 2Pin</t>
   </si>
   <si>
+    <t xml:space="preserve">power in and Run contact</t>
+  </si>
+  <si>
     <t xml:space="preserve">**</t>
   </si>
   <si>
@@ -113,6 +116,12 @@
   </si>
   <si>
     <t xml:space="preserve">Design, Testing and Manufacturing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pin Headers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wires</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -132,7 +141,6 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -155,14 +163,12 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -395,7 +401,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -485,6 +491,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -541,7 +559,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G1048576"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
@@ -549,7 +567,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="22.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="5.99"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="8" style="1" width="10.51"/>
   </cols>
@@ -915,32 +933,25 @@
         <v>3</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18" s="15" t="n">
         <f aca="false">C18*D18</f>
-        <v>3</v>
-      </c>
-      <c r="F18" s="16"/>
+        <v>6</v>
+      </c>
+      <c r="F18" s="16" t="s">
+        <v>27</v>
+      </c>
       <c r="G18" s="18"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>28</v>
-      </c>
+      <c r="A19" s="6"/>
+      <c r="B19" s="13"/>
       <c r="C19" s="14"/>
-      <c r="D19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="15" t="n">
-        <f aca="false">C19*D19</f>
-        <v>0</v>
-      </c>
+      <c r="D19" s="6"/>
+      <c r="E19" s="15"/>
       <c r="F19" s="16"/>
-      <c r="G19" s="17"/>
+      <c r="G19" s="18"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6"/>
@@ -948,52 +959,118 @@
       <c r="C20" s="14"/>
       <c r="D20" s="6"/>
       <c r="E20" s="15"/>
-      <c r="G20" s="17"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="18"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="C21" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="22" t="n">
+      <c r="C21" s="14"/>
+      <c r="D21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="15" t="n">
         <f aca="false">C21*D21</f>
         <v>0</v>
       </c>
       <c r="F21" s="16"/>
       <c r="G21" s="17"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6"/>
-      <c r="B22" s="23"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="16"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="15"/>
       <c r="G22" s="17"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2"/>
-      <c r="B23" s="27" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="28"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="3" t="n">
-        <f aca="false">SUM(E2:E22)</f>
-        <v>660.34</v>
-      </c>
-      <c r="F23" s="30"/>
-      <c r="G23" s="31"/>
-    </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="C23" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="22" t="n">
+        <f aca="false">C23*D23</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="16"/>
+      <c r="G23" s="17"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="23" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="D24" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="15" t="n">
+        <f aca="false">C24*D24</f>
+        <v>10</v>
+      </c>
+      <c r="F24" s="16"/>
+      <c r="G24" s="17"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="23" t="n">
+        <v>19</v>
+      </c>
+      <c r="B25" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" s="25" t="n">
+        <v>6</v>
+      </c>
+      <c r="D25" s="23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E25" s="15" t="n">
+        <f aca="false">C25*D25</f>
+        <v>3</v>
+      </c>
+      <c r="F25" s="16"/>
+      <c r="G25" s="17"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6"/>
+      <c r="B26" s="26"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="28"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="17"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2"/>
+      <c r="B27" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="C27" s="31"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="3" t="n">
+        <f aca="false">SUM(E2:E26)</f>
+        <v>676.34</v>
+      </c>
+      <c r="F27" s="33"/>
+      <c r="G27" s="34"/>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>